<commit_message>
update on negative ionization mode code
</commit_message>
<xml_diff>
--- a/neg_splashlipidomix_list.xlsx
+++ b/neg_splashlipidomix_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saralondonoosorio/Documents/GitHub/CEMBIO-EURAC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64F3D97D-839C-504A-996D-261A316E3750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FFA60D-D8CC-D84E-B4EE-DC2DE9BC6046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29400" yWindow="8420" windowWidth="29400" windowHeight="18380" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
+    <workbookView xWindow="25660" yWindow="660" windowWidth="25380" windowHeight="26400" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
   <si>
     <t>PC</t>
   </si>
@@ -98,14 +98,74 @@
     <t>MG(18:1/0:0(d7))</t>
   </si>
   <si>
-    <t>MG</t>
+    <t>LPI</t>
+  </si>
+  <si>
+    <t>Endogenous</t>
+  </si>
+  <si>
+    <t>FA(22:0)</t>
+  </si>
+  <si>
+    <t>dPI</t>
+  </si>
+  <si>
+    <t>dPE</t>
+  </si>
+  <si>
+    <t>dPC</t>
+  </si>
+  <si>
+    <t>dLPE</t>
+  </si>
+  <si>
+    <t>dLPC</t>
+  </si>
+  <si>
+    <t>dFA</t>
+  </si>
+  <si>
+    <t>dMG</t>
+  </si>
+  <si>
+    <t>HexCer(d42:2)</t>
+  </si>
+  <si>
+    <t>PI(18:0/18:1)</t>
+  </si>
+  <si>
+    <t>PE(16:0/18:1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC(18:1_20:4) </t>
+  </si>
+  <si>
+    <t>LPE(16:0/0:0)</t>
+  </si>
+  <si>
+    <t>Cer(d18:0/24:0)</t>
+  </si>
+  <si>
+    <t>Cer</t>
+  </si>
+  <si>
+    <t>HexCer</t>
+  </si>
+  <si>
+    <t>LPC(0:0/18:1)</t>
+  </si>
+  <si>
+    <t>LPI(18:0/0:0)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -121,13 +181,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -142,13 +213,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,10 +557,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFD69E1-DE54-004B-BA8F-573A6CD4FC04}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1"/>
+    <col min="2" max="2" width="37.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -516,18 +591,18 @@
       <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="4">
         <v>828.5625</v>
       </c>
       <c r="D2" s="3">
         <v>6.37</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E7" si="0">D2*60</f>
+        <f t="shared" ref="E2:E17" si="0">D2*60</f>
         <v>382.2</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -537,7 +612,7 @@
       <c r="B3" t="s">
         <v>11</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="4">
         <v>709.55169999999998</v>
       </c>
       <c r="D3" s="3">
@@ -548,7 +623,7 @@
         <v>512.4</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -558,7 +633,7 @@
       <c r="B4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="4">
         <v>811.61980000000005</v>
       </c>
       <c r="D4" s="3">
@@ -569,7 +644,7 @@
         <v>493.20000000000005</v>
       </c>
       <c r="F4" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -579,7 +654,7 @@
       <c r="B5" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="4">
         <v>485.33780000000002</v>
       </c>
       <c r="D5" s="3">
@@ -590,7 +665,7 @@
         <v>169.8</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -600,7 +675,7 @@
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="4">
         <v>587.4058</v>
       </c>
       <c r="D6" s="3">
@@ -611,7 +686,7 @@
         <v>163.20000000000002</v>
       </c>
       <c r="F6" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -621,18 +696,18 @@
       <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="4">
         <v>286.42750000000001</v>
       </c>
       <c r="D7" s="3">
         <v>3.5209999999999999</v>
       </c>
       <c r="E7">
-        <f>D7*60</f>
+        <f t="shared" si="0"/>
         <v>211.26</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -642,18 +717,207 @@
       <c r="B8" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="4">
         <v>422.3503</v>
       </c>
       <c r="D8">
         <v>3.65</v>
       </c>
       <c r="E8">
-        <f>D8*60</f>
+        <f t="shared" si="0"/>
         <v>219</v>
       </c>
       <c r="F8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="4">
+        <v>710.66669999999999</v>
+      </c>
+      <c r="D9" s="3">
+        <v>12.69</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>761.4</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="4">
+        <v>339.3268314124</v>
+      </c>
+      <c r="D10">
+        <v>6.34</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>380.4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="4">
+        <v>868.68827192109995</v>
+      </c>
+      <c r="D11">
+        <v>11.97</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>718.2</v>
+      </c>
+      <c r="F11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="4">
+        <v>599.32016833329999</v>
+      </c>
+      <c r="D12">
+        <v>2.84</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>170.39999999999998</v>
+      </c>
+      <c r="F12" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="4">
+        <v>863.56548436050002</v>
+      </c>
+      <c r="D13">
+        <v>8.67</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>520.20000000000005</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="4">
+        <v>866.59159999999997</v>
+      </c>
+      <c r="D14">
+        <v>8.1199999999999992</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>487.19999999999993</v>
+      </c>
+      <c r="F14" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="4">
+        <v>580.36194230119997</v>
+      </c>
+      <c r="D15">
+        <v>2.56</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="0"/>
+        <v>153.6</v>
+      </c>
+      <c r="F15" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="4">
+        <v>716.52355807159995</v>
+      </c>
+      <c r="D16">
+        <v>9.82</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="0"/>
+        <v>589.20000000000005</v>
+      </c>
+      <c r="F16" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="4">
+        <v>452.27820000000003</v>
+      </c>
+      <c r="D17">
+        <v>2.67</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>160.19999999999999</v>
+      </c>
+      <c r="F17" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new compounds on IS_neg
</commit_message>
<xml_diff>
--- a/neg_splashlipidomix_list.xlsx
+++ b/neg_splashlipidomix_list.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saralondonoosorio/Documents/GitHub/CEMBIO-EURAC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37FFA60D-D8CC-D84E-B4EE-DC2DE9BC6046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D1B4F3-9A9F-FD47-9191-1E444CC8F9E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25660" yWindow="660" windowWidth="25380" windowHeight="26400" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{9E5E902E-872A-BE45-A1A9-54571E2C3B45}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$22</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="50">
   <si>
     <t>PC</t>
   </si>
@@ -156,6 +159,36 @@
   </si>
   <si>
     <t>LPI(18:0/0:0)</t>
+  </si>
+  <si>
+    <t>PC(18:0/18:2)</t>
+  </si>
+  <si>
+    <t>Pcnew</t>
+  </si>
+  <si>
+    <t>PC(16:0/18:2)</t>
+  </si>
+  <si>
+    <t>PCnew2</t>
+  </si>
+  <si>
+    <t>LPCnew</t>
+  </si>
+  <si>
+    <t>LPInew</t>
+  </si>
+  <si>
+    <t>LPC(18:0/0:0)</t>
+  </si>
+  <si>
+    <t>LPI(20:4/0:0)</t>
+  </si>
+  <si>
+    <t>PInew</t>
+  </si>
+  <si>
+    <t>PI(18:0/18:2)</t>
   </si>
 </sst>
 </file>
@@ -187,7 +220,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -197,6 +230,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -213,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -223,6 +262,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -557,7 +597,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFD69E1-DE54-004B-BA8F-573A6CD4FC04}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.83203125" customWidth="1"/>
@@ -586,65 +626,65 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
+        <v>21</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="C2" s="4">
-        <v>828.5625</v>
-      </c>
-      <c r="D2" s="3">
-        <v>6.37</v>
+        <v>619.28890000000001</v>
+      </c>
+      <c r="D2">
+        <v>1.64</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E17" si="0">D2*60</f>
-        <v>382.2</v>
+        <f>D2*60</f>
+        <v>98.399999999999991</v>
       </c>
       <c r="F2" t="s">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
+        <v>21</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>38</v>
       </c>
       <c r="C3" s="4">
-        <v>709.55169999999998</v>
-      </c>
-      <c r="D3" s="3">
-        <v>8.5399999999999991</v>
+        <v>580.36194230119997</v>
+      </c>
+      <c r="D3">
+        <v>2.56</v>
       </c>
       <c r="E3">
-        <f t="shared" si="0"/>
-        <v>512.4</v>
+        <f>D3*60</f>
+        <v>153.6</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C4" s="4">
-        <v>811.61980000000005</v>
-      </c>
-      <c r="D4" s="3">
-        <v>8.2200000000000006</v>
+        <v>452.27820000000003</v>
+      </c>
+      <c r="D4">
+        <v>2.67</v>
       </c>
       <c r="E4">
-        <f t="shared" si="0"/>
-        <v>493.20000000000005</v>
+        <f>D4*60</f>
+        <v>160.19999999999999</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -652,20 +692,20 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5" s="4">
-        <v>485.33780000000002</v>
+        <v>587.4058</v>
       </c>
       <c r="D5" s="3">
-        <v>2.83</v>
+        <v>2.72</v>
       </c>
       <c r="E5">
-        <f t="shared" si="0"/>
-        <v>169.8</v>
+        <f>D5*60</f>
+        <v>163.20000000000002</v>
       </c>
       <c r="F5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -673,104 +713,104 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="4">
-        <v>587.4058</v>
+        <v>485.33780000000002</v>
       </c>
       <c r="D6" s="3">
-        <v>2.72</v>
+        <v>2.83</v>
       </c>
       <c r="E6">
-        <f t="shared" si="0"/>
-        <v>163.20000000000002</v>
+        <f>D6*60</f>
+        <v>169.8</v>
       </c>
       <c r="F6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>15</v>
+        <v>21</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>39</v>
       </c>
       <c r="C7" s="4">
-        <v>286.42750000000001</v>
-      </c>
-      <c r="D7" s="3">
-        <v>3.5209999999999999</v>
+        <v>599.32016833329999</v>
+      </c>
+      <c r="D7">
+        <v>2.84</v>
       </c>
       <c r="E7">
-        <f t="shared" si="0"/>
-        <v>211.26</v>
+        <f>D7*60</f>
+        <v>170.39999999999998</v>
       </c>
       <c r="F7" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>46</v>
       </c>
       <c r="C8" s="4">
-        <v>422.3503</v>
+        <v>582.37760000000003</v>
       </c>
       <c r="D8">
-        <v>3.65</v>
+        <v>3.44</v>
       </c>
       <c r="E8">
-        <f t="shared" si="0"/>
-        <v>219</v>
+        <f>D8*60</f>
+        <v>206.4</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C9" s="4">
-        <v>710.66669999999999</v>
+        <v>286.42750000000001</v>
       </c>
       <c r="D9" s="3">
-        <v>12.69</v>
+        <v>3.5209999999999999</v>
       </c>
       <c r="E9">
-        <f t="shared" si="0"/>
-        <v>761.4</v>
+        <f>D9*60</f>
+        <v>211.26</v>
       </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4">
-        <v>339.3268314124</v>
+        <v>422.3503</v>
       </c>
       <c r="D10">
-        <v>6.34</v>
+        <v>3.65</v>
       </c>
       <c r="E10">
-        <f t="shared" si="0"/>
-        <v>380.4</v>
+        <f>D10*60</f>
+        <v>219</v>
       </c>
       <c r="F10" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -778,41 +818,41 @@
         <v>21</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C11" s="4">
-        <v>868.68827192109995</v>
+        <v>339.3268314124</v>
       </c>
       <c r="D11">
-        <v>11.97</v>
+        <v>6.34</v>
       </c>
       <c r="E11">
-        <f t="shared" si="0"/>
-        <v>718.2</v>
+        <f>D11*60</f>
+        <v>380.4</v>
       </c>
       <c r="F11" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>39</v>
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>10</v>
       </c>
       <c r="C12" s="4">
-        <v>599.32016833329999</v>
-      </c>
-      <c r="D12">
-        <v>2.84</v>
+        <v>828.5625</v>
+      </c>
+      <c r="D12" s="3">
+        <v>6.37</v>
       </c>
       <c r="E12">
-        <f t="shared" si="0"/>
-        <v>170.39999999999998</v>
+        <f>D12*60</f>
+        <v>382.2</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -820,20 +860,20 @@
         <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C13" s="4">
-        <v>863.56548436050002</v>
+        <v>861.5498</v>
       </c>
       <c r="D13">
-        <v>8.67</v>
+        <v>7.46</v>
       </c>
       <c r="E13">
-        <f t="shared" si="0"/>
-        <v>520.20000000000005</v>
+        <f>D13*60</f>
+        <v>447.6</v>
       </c>
       <c r="F13" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -841,86 +881,196 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="C14" s="4">
-        <v>866.59159999999997</v>
+        <v>816.57600000000002</v>
       </c>
       <c r="D14">
-        <v>8.1199999999999992</v>
+        <v>7.91</v>
       </c>
       <c r="E14">
-        <f t="shared" si="0"/>
-        <v>487.19999999999993</v>
+        <f>D14*60</f>
+        <v>474.6</v>
       </c>
       <c r="F14" t="s">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>21</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>38</v>
+      <c r="B15" t="s">
+        <v>33</v>
       </c>
       <c r="C15" s="4">
-        <v>580.36194230119997</v>
+        <v>866.59159999999997</v>
       </c>
       <c r="D15">
-        <v>2.56</v>
+        <v>8.1199999999999992</v>
       </c>
       <c r="E15">
-        <f t="shared" si="0"/>
-        <v>153.6</v>
+        <f>D15*60</f>
+        <v>487.19999999999993</v>
       </c>
       <c r="F15" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C16" s="4">
-        <v>716.52355807159995</v>
-      </c>
-      <c r="D16">
-        <v>9.82</v>
+        <v>811.61980000000005</v>
+      </c>
+      <c r="D16" s="3">
+        <v>8.2200000000000006</v>
       </c>
       <c r="E16">
-        <f t="shared" si="0"/>
-        <v>589.20000000000005</v>
+        <f>D16*60</f>
+        <v>493.20000000000005</v>
       </c>
       <c r="F16" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B17" t="s">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="C17" s="4">
-        <v>452.27820000000003</v>
-      </c>
-      <c r="D17">
-        <v>2.67</v>
+        <v>709.55169999999998</v>
+      </c>
+      <c r="D17" s="3">
+        <v>8.5399999999999991</v>
       </c>
       <c r="E17">
-        <f t="shared" si="0"/>
-        <v>160.19999999999999</v>
+        <f>D17*60</f>
+        <v>512.4</v>
       </c>
       <c r="F17" t="s">
-        <v>17</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="4">
+        <v>863.56548436050002</v>
+      </c>
+      <c r="D18">
+        <v>8.67</v>
+      </c>
+      <c r="E18">
+        <f>D18*60</f>
+        <v>520.20000000000005</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="4">
+        <v>716.52355807159995</v>
+      </c>
+      <c r="D19">
+        <v>9.82</v>
+      </c>
+      <c r="E19">
+        <f>D19*60</f>
+        <v>589.20000000000005</v>
+      </c>
+      <c r="F19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="4">
+        <v>844.60730000000001</v>
+      </c>
+      <c r="D20">
+        <v>10.01</v>
+      </c>
+      <c r="E20">
+        <f>D20*60</f>
+        <v>600.6</v>
+      </c>
+      <c r="F20" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="4">
+        <v>868.68827192109995</v>
+      </c>
+      <c r="D21">
+        <v>11.97</v>
+      </c>
+      <c r="E21">
+        <f>D21*60</f>
+        <v>718.2</v>
+      </c>
+      <c r="F21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="4">
+        <v>710.66669999999999</v>
+      </c>
+      <c r="D22" s="3">
+        <v>12.69</v>
+      </c>
+      <c r="E22">
+        <f>D22*60</f>
+        <v>761.4</v>
+      </c>
+      <c r="F22" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F22" xr:uid="{5BFD69E1-DE54-004B-BA8F-573A6CD4FC04}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F22">
+      <sortCondition ref="E1:E22"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>